<commit_message>
Ajout répertoire PDF + metadata fsh 1a30e17ed58891b09634e7f665f5dde139d2f752
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgc-metadata.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgc-metadata.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="88">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-15T13:41:49+00:00</t>
+    <t>2026-07-15T16:11:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,8 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Le fichier METADATA.XML porte les métadonnées des documents cliniques d'un patient</t>
+    <t>Modèle logique décrivant la structure d'un fichier METADATA associé à un SUBSET IHE XDM.
+Regroupe un SubmissionSet, ses DocumentEntries et les Associations entre objets.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -243,7 +244,44 @@
     <t>*</t>
   </si>
   <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
     <t>Base</t>
+  </si>
+  <si>
+    <t>pdlgc-metadata.submissionSet</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/SubmissionSet
+</t>
+  </si>
+  <si>
+    <t>Lot de soumission du SUBSET</t>
+  </si>
+  <si>
+    <t>pdlgc-metadata.documentEntry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/DocumentEntry
+</t>
+  </si>
+  <si>
+    <t>Fiches documentaires des documents inclus dans le SUBSET</t>
+  </si>
+  <si>
+    <t>pdlgc-metadata.association</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/association-xdm
+</t>
+  </si>
+  <si>
+    <t>Associations entre objets du SUBSET (remplacement, transformation)</t>
   </si>
 </sst>
 </file>
@@ -545,11 +583,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ2"/>
+  <dimension ref="A1:AJ5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="13.375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="13.375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="25.984375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="25.984375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -558,7 +596,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="7.6796875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="62.890625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -579,7 +617,7 @@
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="9.91015625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="25.984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
@@ -723,7 +761,7 @@
         <v>73</v>
       </c>
       <c r="K2" t="s" s="2">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L2" t="s" s="2">
         <v>9</v>
@@ -780,7 +818,7 @@
         <v>73</v>
       </c>
       <c r="AF2" t="s" s="2">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AG2" t="s" s="2">
         <v>74</v>
@@ -792,6 +830,306 @@
         <v>73</v>
       </c>
       <c r="AJ2" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G3" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K3" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="L3" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="M3" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q3" s="2"/>
+      <c r="R3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AG3" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH3" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI3" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ3" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G4" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K4" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="L4" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="M4" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q4" s="2"/>
+      <c r="R4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF4" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AG4" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH4" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ4" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G5" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K5" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="L5" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="M5" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q5" s="2"/>
+      <c r="R5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF5" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AG5" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH5" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ5" t="s" s="2">
         <v>73</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Maje des FSH XDM pour la convention de nommage 0662327b4c8e0a86dd103a35731d079c758073ac
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgc-metadata.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgc-metadata.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-17T14:49:58+00:00</t>
+    <t>2026-07-19T17:20:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -257,7 +257,7 @@
     <t>1</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/SubmissionSet
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdm-submission-set
 </t>
   </si>
   <si>
@@ -267,7 +267,7 @@
     <t>pdlgc-metadata.documentEntry</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/DocumentEntry
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdm-document-entry
 </t>
   </si>
   <si>
@@ -277,7 +277,7 @@
     <t>pdlgc-metadata.association</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/association-xdm
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdm-association
 </t>
   </si>
   <si>
@@ -596,7 +596,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="62.890625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="66.70703125" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>